<commit_message>
Extract lab flags + bare reference ranges, add PCV (BM046), findings summary with lab interpretation
- parse_service: optional (ABBR) between biomarker name and value
  (Hemoglobin (Hb) 12.5), bare 'lo - hi' reference ranges
  (13.0 - 17.0, 4000-11000), lab flag capture (Low/High/Borderline),
  extract_interpretation() for the lab's Interpretation line
- analysis_service: findings-style summary listing each out-of-range
  result with value/range/lab flag, quotes lab interpretation,
  educational disclaimer; flag transcribed to status when no range
- spec: add Packed Cell Volume / PCV / Hematocrit / HCT as BM046
  (xlsx source of truth + regenerated biomarkers.json)
- API: Result.flag persisted (ensure_columns backfills older DBs),
  summary includes interpretation
- frontend: new Lab flag column in results table
- tests: 64 passing; eval extraction/classification/trends still 1.0
</commit_message>
<xml_diff>
--- a/data/biomarkers/BloodIQ_Biomarker_Specification_v2.xlsx
+++ b/data/biomarkers/BloodIQ_Biomarker_Specification_v2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biomarkers" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Notes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Biomarkers" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Implementation Notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Biomarkers'!$A$1:$I$46</definedName>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2602,6 +2602,53 @@
       <c r="I46" t="inlineStr">
         <is>
           <t>May be reported with an equation or calculation method; do not treat as an ordinary analyte reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>BM046</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Packed Cell Volume</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>CBC / Hematology</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>PCV, Packed Cell Volume, Hematocrit, HCT</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Proportion of blood volume occupied by red blood cells</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range; preserve original unit.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
match test2's printed names: Fasting Blood Sugar, Direct LDL; veto ratios
Live AI run showed two matcher gaps: 'Fasting Blood Sugar' didn't map
to Glucose (row dropped) and 'Direct LDL' didn't map to LDL, while
'LDL/HDL Ratio' wrongly merged into LDL. Added the aliases to the xlsx
source of truth + regenerated biomarkers.json, and added 'ratio' to the
subtype-qualifier veto list. Formal eval still 1.0 across the board.
</commit_message>
<xml_diff>
--- a/data/biomarkers/BloodIQ_Biomarker_Specification_v2.xlsx
+++ b/data/biomarkers/BloodIQ_Biomarker_Specification_v2.xlsx
@@ -978,7 +978,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Blood Glucose, Fasting Glucose, Serum Glucose</t>
+          <t>Blood Glucose, Fasting Glucose, Serum Glucose, Fasting Blood Sugar, FBS, Blood Sugar</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1777,7 +1777,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>LDL-C, LDL Cholesterol, Low-Density Lipoprotein</t>
+          <t>LDL-C, LDL Cholesterol, Low-Density Lipoprotein, Direct LDL</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">

</xml_diff>

<commit_message>
Add Alpha Fetoprotein (AFP) to the biomarker spec (BM047)
Single-test reports like Ram's Alfa Laboratories AFP scan returned 0
biomarkers because AFP was not in the 46-marker spec. Added BM047 with
aliases (AFP, Alpha Feto Protein, Alpha-Fetoprotein) to the xlsx source
of truth and regenerated biomarkers.json (47 markers). Updated the two
spec-count tests and added an AFP alias-mapping test.
</commit_message>
<xml_diff>
--- a/data/biomarkers/BloodIQ_Biomarker_Specification_v2.xlsx
+++ b/data/biomarkers/BloodIQ_Biomarker_Specification_v2.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2647,6 +2647,53 @@
         </is>
       </c>
       <c r="I47" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range; preserve original unit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>BM047</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Alpha Fetoprotein</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Tumor Markers / Immunology</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>AFP, Alpha Feto Protein, Alpha-Fetoprotein, Alpha Fetoprotein</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>ng/mL</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Protein produced mainly by the fetal liver; measured in adults as a tumor marker</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
         <is>
           <t>Use report-specific reference range; preserve original unit.</t>
         </is>

</xml_diff>

<commit_message>
Expand biomarker spec 47 -> 146 from MedlinePlus lab-tests index
- 99 new markers (BM048-BM146) across 12 categories: Urinalysis (17),
  Stool (4), Semen (3), Hormones (16), Cardiac (4), Coagulation (6),
  Diabetes (1), Infection/Immune/Autoimmune (9), Thyroid (5),
  Tumor markers (6), CBC differential + MPV (6), Blood gas (3),
  CSF (3), Metabolic/Pancreatic/Liver/Toxicology (16).
- Narrative/imaging/procedure/qualitative-infectious tests (ultrasound,
  PET, biopsies, cultures, genetic tests, ECG...) deliberately excluded.
- Aliases verified collision-free; urine-vs-serum disambiguation
  confirmed via the subtype-qualifier matcher (22/22 correct).
- xlsx remains source of truth; JSON regenerated via import_spec.
</commit_message>
<xml_diff>
--- a/data/biomarkers/BloodIQ_Biomarker_Specification_v2.xlsx
+++ b/data/biomarkers/BloodIQ_Biomarker_Specification_v2.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2696,6 +2696,4607 @@
       <c r="I48" t="inlineStr">
         <is>
           <t>Use report-specific reference range; preserve original unit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>BM048</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Urine pH</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Urinalysis</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Urine pH, pH Urine, Urine PH</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Acidity/alkalinity of urine</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Dipstick or meter reading; use report-specific range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>BM049</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Urine Specific Gravity</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Urinalysis</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Specific Gravity, Urine Specific Gravity, Sp Gr, SG Urine</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Concentration of dissolved particles in urine</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>BM050</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Urine Protein</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Urinalysis</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Urine Protein, Protein Urine, Proteinuria</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>mg/dL</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Protein excreted in urine; marker of kidney stress</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Dipstick bands are ordinal; preserve the printed value as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>BM051</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Urine Glucose</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Urinalysis</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Urine Glucose, Glucose Urine, Glycosuria</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>mg/dL</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Glucose spilling into urine</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Dipstick bands are ordinal; preserve the printed value as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>BM052</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Urine Ketones</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Urinalysis</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Urine Ketones, Ketones Urine, Ketone Bodies Urine</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Ketone bodies in urine</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Dipstick bands are ordinal (negative/trace/small/moderate/large).</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>BM053</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Urine Bilirubin</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Urinalysis</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Urine Bilirubin, Bilirubin Urine</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Bilirubin detected in urine</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Dipstick qualitative result; do not trend numerically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>BM054</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Urine Urobilinogen</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Urinalysis</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Urine Urobilinogen, Urobilinogen Urine</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>mg/dL</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Urobilinogen level in urine</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>BM055</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Urine Blood</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Urinalysis</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Urine Blood, Blood Urine, Hematuria</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Blood detected in urine</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Dipstick qualitative result; do not trend numerically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>BM056</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Urine Nitrite</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Urinalysis</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Urine Nitrite, Nitrite Urine, Nitrites</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Nitrite in urine; bacterial marker</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Qualitative result; do not trend numerically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>BM057</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Urine Leukocyte Esterase</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Urinalysis</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Urine Leukocyte Esterase, Leukocyte Esterase Urine, LE Urine</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>White-cell enzyme in urine; inflammation marker</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Qualitative result; do not trend numerically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>BM058</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Urine Calcium</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Urinalysis</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Urine Calcium, Calcium Urine, 24h Urine Calcium</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>mg/24h</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Calcium excreted in urine over 24 hours</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>BM059</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Urine Phosphate</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Urinalysis</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Urine Phosphate, Phosphate Urine, Phosphorus Urine</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>mg/24h</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Phosphate excreted in urine over 24 hours</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>BM060</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Microalbumin/Creatinine Ratio</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Urinalysis</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Microalbumin Creatinine Ratio, Albumin Creatinine Ratio, ACR, Microalbumin/Cr</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>mg/g</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Urine albumin normalized to creatinine; early kidney-damage screen</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Key diabetes kidney screen; use report-specific range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>BM061</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Urine Osmolality</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Urinalysis</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Urine Osmolality, Osmolality Urine</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>mOsm/kg</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Concentration of urine solutes</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>BM062</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Urine Epithelial Cells</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Urinalysis</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Urine Epithelial Cells, Epithelial Cells Urine</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>/hpf</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Epithelial cells seen on urine microscopy</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Microscopy ordinal result (rare/few/moderate/many); do not trend numerically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>BM063</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Urine Mucus</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Urinalysis</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Urine Mucus, Mucus Urine</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Mucus threads seen on urine microscopy</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Microscopy ordinal result; do not trend numerically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>BM064</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Urine Crystals</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Urinalysis</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Urine Crystals, Crystals Urine</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Crystals seen on urine microscopy</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Microscopy descriptive result; do not trend numerically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>BM065</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Fecal Calprotectin</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Stool</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Calprotectin, Fecal Calprotectin, Stool Calprotectin</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>µg/g</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Intestinal inflammation marker in stool</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>BM066</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Fecal Occult Blood</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Stool</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>FOBT, Fecal Occult Blood, Occult Blood Stool, FIT Test</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Hidden blood in stool; colorectal screen</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Qualitative result; do not trend numerically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>BM067</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Fecal Elastase</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Stool</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Elastase, Fecal Elastase, Stool Elastase, Pancreatic Elastase</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>µg/g</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Pancreatic enzyme output marker</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>BM068</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Fecal Chymotrypsin</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Stool</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Chymotrypsin, Fecal Chymotrypsin, Stool Chymotrypsin</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>U/g</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Pancreatic digestive enzyme in stool</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>BM069</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Sperm Concentration</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Semen</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Sperm Count, Sperm Concentration, Sperm Density</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>million/mL</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Number of sperm per milliliter of semen</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>BM070</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Sperm Motility</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Semen</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Motility, Sperm Motility, Progressive Motility</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Share of moving sperm</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>BM071</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Sperm Morphology</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Semen</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Morphology, Sperm Morphology, Normal Forms</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Share of normally shaped sperm</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>BM072</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>ACTH</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Hormones</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>ACTH, Adrenocorticotropic Hormone, Corticotropin</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>pg/mL</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Pituitary hormone driving cortisol release</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Time-of-day matters; use report-specific range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>BM073</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Aldosterone</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Hormones</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Aldosterone</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ng/dL</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Adrenal hormone regulating salt and blood pressure</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>BM074</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Cortisol</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Hormones</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Cortisol, Serum Cortisol</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>µg/dL</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Adrenal stress hormone</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Time-of-day matters; use report-specific range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>BM075</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>DHEA-S</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Hormones</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>DHEA-S, DHEA Sulfate, Dehydroepiandrosterone Sulfate</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>µg/dL</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Adrenal androgen precursor</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Age- and sex-dependent; use report-specific range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>BM076</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Testosterone</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Hormones</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Testosterone, Total Testosterone</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ng/dL</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Primary male sex hormone</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Sex-dependent; use report-specific range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>BM077</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Estradiol</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Hormones</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Estradiol, Estrogen, E2</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>pg/mL</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Primary estrogen hormone</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Cycle/menopause-dependent; use report-specific range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>BM078</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Progesterone</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Hormones</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Progesterone</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ng/mL</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Ovarian hormone of the menstrual cycle and pregnancy</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Cycle/pregnancy-dependent; use report-specific range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>BM079</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Prolactin</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Hormones</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Prolactin, PRL</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ng/mL</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Pituitary hormone for lactation</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>BM080</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>LH</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Hormones</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>LH, Luteinizing Hormone</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>mIU/mL</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Pituitary reproductive hormone</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Cycle-dependent; use report-specific range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>BM081</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>FSH</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Hormones</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>FSH, Follicle-Stimulating Hormone</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>mIU/mL</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Pituitary reproductive hormone</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Cycle/menopause-dependent; use report-specific range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>BM082</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>AMH</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Hormones</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>AMH, Anti-Mullerian Hormone, Anti-Müllerian Hormone</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>ng/mL</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Ovarian reserve marker</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>BM083</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>PTH</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Hormones</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>PTH, Parathyroid Hormone, Intact PTH</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>pg/mL</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Calcium-regulating parathyroid hormone</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>BM084</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Calcitonin</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Hormones</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Calcitonin</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>pg/mL</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Thyroid C-cell hormone; medullary thyroid marker</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>BM085</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>17-Hydroxyprogesterone</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Hormones</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>17-Hydroxyprogesterone, 17-OHP, 17 OH Progesterone</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>ng/dL</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Adrenal steroid pathway marker</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>BM086</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>SHBG</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Hormones</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>SHBG, Sex Hormone Binding Globulin</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>nmol/L</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Protein binding sex hormones in blood</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>BM087</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Renin</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Hormones</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Renin, Plasma Renin</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>ng/mL/h</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Kidney enzyme starting blood-pressure regulation</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Posture/salt-dependent; use report-specific range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>BM088</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Troponin I</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Cardiac</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Troponin I, Troponin, cTnI, High Sensitivity Troponin</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>ng/mL</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Heart-muscle injury marker</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Assay-dependent cutoffs; use report-specific range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>BM089</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>NT-proBNP</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Cardiac</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>NT-proBNP, NT proBNP, ProBNP</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>pg/mL</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Heart-failure stretch marker</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Age-dependent; use report-specific range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>BM090</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Creatine Kinase</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Cardiac / Muscle</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>CK, Creatine Kinase, CPK, Creatine Phosphokinase</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>U/L</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Muscle-damage enzyme</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>BM091</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>LDH</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Enzymes</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>LDH, Lactate Dehydrogenase</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>U/L</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Tissue-turnover enzyme</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>BM092</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>PT/INR</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Coagulation</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>PT INR, Prothrombin Time, INR, PT/INR</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Blood clotting time standardized as INR</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Therapeutic target depends on indication; use report range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>BM093</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>PTT</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Coagulation</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>PTT, Partial Thromboplastin Time, aPTT, APTT</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>sec</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Intrinsic clotting pathway time</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>BM094</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>D-Dimer</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Coagulation</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>D-Dimer, D Dimer, DDimer</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>ng/mL</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Clot-breakdown fragment; clot screen</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Assay-dependent cutoff; use report-specific range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>BM095</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Fibrinogen</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Coagulation</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Fibrinogen</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>mg/dL</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Clotting protein made by the liver</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>BM096</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Protein C</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Coagulation</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Protein C</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Natural anticoagulant protein activity</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>BM097</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Protein S</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Coagulation</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Protein S, Free Protein S</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Natural anticoagulant protein activity</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>BM098</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>C-Peptide</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Diabetes</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>C-Peptide, C Peptide, Connecting Peptide</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>ng/mL</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Insulin-production marker</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>BM099</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Procalcitonin</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Infection</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Procalcitonin, PCT</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>ng/mL</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Bacterial-infection marker</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>BM100</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Haptoglobin</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>CBC / Hematology</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Haptoglobin, HP</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>mg/dL</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Hemoglobin-scavenging protein; hemolysis marker</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>BM101</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Complement C3</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Immune</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>C3, Complement C3</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>mg/dL</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Immune-system complement protein</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>BM102</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Complement C4</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Immune</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>C4, Complement C4</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>mg/dL</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Immune-system complement protein</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>BM103</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>CD4 Count</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Immune</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>CD4, CD4 Count, CD4 Lymphocyte Count</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>cells/µL</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Helper T-cell count; immune status marker</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>BM104</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Total IgE</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Immune</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>IgE, Total IgE, Immunoglobulin E</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>IU/mL</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Allergy-related antibody level</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>BM105</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Rheumatoid Factor</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Autoimmune</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>RF, Rheumatoid Factor</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>IU/mL</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Autoantibody linked to rheumatoid arthritis</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>BM106</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Anti-CCP</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Autoimmune</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>CCP, Anti-CCP, Anti CCP, Cyclic Citrullinated Peptide</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>U/mL</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Rheumatoid arthritis autoantibody</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>BM107</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>ANA</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Autoimmune</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>ANA, Antinuclear Antibody</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>titer</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Antinuclear antibody screen titer</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Titer + pattern result; do not trend numerically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>BM108</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Free T3</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Thyroid</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Free T3, FT3, Free Triiodothyronine</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>pg/mL</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Active unbound thyroid hormone</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>BM109</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Total T3</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Thyroid</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Total T3, T3, Triiodothyronine</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>ng/dL</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Total triiodothyronine in blood</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>BM110</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>TPO Antibody</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Thyroid</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>TPOAb, TPO Antibody, Anti-TPO, Thyroid Peroxidase Antibody</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>IU/mL</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Autoimmune thyroid antibody</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>BM111</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Thyroglobulin Antibody</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Thyroid</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>TgAb, Thyroglobulin Antibody, Anti-Thyroglobulin</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>IU/mL</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Autoimmune thyroid antibody</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>BM112</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Thyroglobulin</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Thyroid</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Thyroglobulin, Tg</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>ng/mL</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Thyroid protein; cancer follow-up marker</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>BM113</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>CA 19-9</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Tumor Markers / Immunology</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>CA 19-9, CA19-9, CA 199</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>U/mL</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Pancreatic/gastrointestinal tumor marker</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>BM114</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>CA-125</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Tumor Markers / Immunology</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>CA-125, CA125</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>U/mL</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Ovarian tumor marker</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>BM115</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>CEA</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Tumor Markers / Immunology</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>CEA, Carcinoembryonic Antigen</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>ng/mL</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Colorectal tumor marker</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Smoking raises baseline; use report-specific range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>BM116</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Beta-2 Microglobulin</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Tumor Markers / Immunology</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>B2M, Beta-2 Microglobulin, Beta 2 Microglobulin</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>mg/L</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Cell-turnover tumor marker</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>BM117</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Kappa Free Light Chains</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Tumor Markers / Immunology</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Kappa Free Light Chains, Kappa FLC, Free Kappa</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>mg/L</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Plasma-cell disorder marker</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>BM118</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Lambda Free Light Chains</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Tumor Markers / Immunology</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Lambda Free Light Chains, Lambda FLC, Free Lambda</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>mg/L</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Plasma-cell disorder marker</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>BM119</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Neutrophils</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>CBC / Hematology</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Neutrophils, Neutrophil %, NEUT, Segs</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Most common infection-fighting white cells</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>BM120</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Lymphocytes</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>CBC / Hematology</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Lymphocytes, Lymphocyte %, LYMPH</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Viral-defense white blood cells</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>BM121</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Monocytes</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>CBC / Hematology</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Monocytes, Monocyte %, MONO</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Tissue-cleanup white blood cells</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>BM122</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Eosinophils</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>CBC / Hematology</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Eosinophils, Eosinophil %, EOS</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Allergy/parasite white blood cells</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>BM123</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Basophils</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>CBC / Hematology</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Basophils, Basophil %, BASO</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Inflammatory white blood cells</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>BM124</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>MPV</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>CBC / Hematology</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>MPV, Mean Platelet Volume</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>fL</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Average platelet size</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>BM125</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Arterial pH</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Blood Gas</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Arterial pH, ABG pH</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr"/>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Blood acidity from arterial sample</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>BM126</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Arterial pCO2</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Blood Gas</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>pCO2, Arterial pCO2, ABG pCO2</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>mmHg</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Arterial carbon dioxide pressure</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>BM127</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Arterial pO2</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Blood Gas</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>pO2, Arterial pO2, ABG pO2, PaO2</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>mmHg</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Arterial oxygen pressure</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>BM128</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>CSF Protein</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Cerebrospinal Fluid</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>CSF Protein, Cerebrospinal Fluid Protein</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>mg/dL</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Protein in cerebrospinal fluid</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>BM129</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>CSF Glucose</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Cerebrospinal Fluid</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>CSF Glucose, Cerebrospinal Fluid Glucose</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>mg/dL</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Glucose in cerebrospinal fluid</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>BM130</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>CSF WBC</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Cerebrospinal Fluid</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>CSF WBC, CSF White Blood Cells, CSF Cell Count</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>/µL</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>White cells in cerebrospinal fluid</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>BM131</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Anion Gap</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Metabolic / Electrolytes</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Anion Gap</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>mEq/L</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Unmeasured-ion gap from electrolytes</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Calculated: Na - (Cl + HCO3)</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Derived from the report's own electrolyte values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>BM132</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Ammonia</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Metabolic / Electrolytes</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Ammonia, Blood Ammonia, NH3</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>µmol/L</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Blood ammonia level</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>BM133</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Serum Osmolality</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Metabolic / Electrolytes</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Serum Osmolality, Osmolality Serum</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>mOsm/kg</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Solute concentration of blood serum</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>BM134</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>GGT</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Liver / Protein</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>GGT, Gamma-GT, Gamma Glutamyl Transferase, Gamma-Glutamyl Transpeptidase</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>U/L</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Liver/bile-duct enzyme</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>BM135</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Globulin</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Liver / Protein</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Globulin, Serum Globulin</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>g/dL</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Non-albumin blood proteins</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Calculated: Total Protein - Albumin</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>Derived from the report's own protein values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>BM136</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>A/G Ratio</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Liver / Protein</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>A/G Ratio, Albumin/Globulin Ratio, Albumin Globulin Ratio</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Albumin to globulin balance</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Calculated: Albumin / Globulin</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>Derived from the report's own protein values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>BM137</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Amylase</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Pancreatic</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Amylase, Serum Amylase</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>U/L</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Pancreatic digestive enzyme</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>BM138</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Lipase</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Pancreatic</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Lipase, Serum Lipase</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>U/L</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>Pancreatic fat-digesting enzyme</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>BM139</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Ceruloplasmin</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Metabolic</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Ceruloplasmin</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>mg/dL</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Copper-carrying blood protein</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>BM140</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Homocysteine</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Metabolic</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Homocysteine</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>µmol/L</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Cardiovascular-risk amino acid</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>BM141</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Methylmalonic Acid</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Vitamins / Nutrition</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>MMA, Methylmalonic Acid, Methylmalonate</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>nmol/L</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Functional B12-deficiency marker</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>BM142</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Prealbumin</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Vitamins / Nutrition</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Prealbumin, Transthyretin</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>mg/dL</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Short-term nutrition status protein</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>BM143</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Sweat Chloride</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Sweat Chloride, Chloride Sweat Test</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>mmol/L</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Sweat chloride; cystic fibrosis screen</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>BM144</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Blood Lead</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Toxicology</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Lead, Blood Lead, Lead Level</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>µg/dL</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Blood lead concentration</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>BM145</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Acetaminophen</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Toxicology</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Acetaminophen, Paracetamol, APAP</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>µg/mL</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Acetaminophen drug level</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>Timing post-dose matters; use report-specific range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>BM146</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Salicylates</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Toxicology</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Salicylates, Salicylate Level, Aspirin Level</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>mg/dL</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Salicylate drug level</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Direct measurement</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>Use report-specific reference range.</t>
         </is>
       </c>
     </row>

</xml_diff>